<commit_message>
Add GIRO and MPACK workflows with dynamic template handling
</commit_message>
<xml_diff>
--- a/resources/rules/Giro.xlsx
+++ b/resources/rules/Giro.xlsx
@@ -7,16 +7,14 @@
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
-    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
-    <sheet name="Лист3" sheetId="3" r:id="rId3"/>
+    <sheet name="Giro" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>Material Description</t>
   </si>
@@ -64,6 +62,60 @@
   </si>
   <si>
     <t>Green</t>
+  </si>
+  <si>
+    <t>Ess Oranges</t>
+  </si>
+  <si>
+    <t>Ess Lemons 12X7</t>
+  </si>
+  <si>
+    <t>Ess Oranges 12X7</t>
+  </si>
+  <si>
+    <t>Ess Lemons</t>
+  </si>
+  <si>
+    <t>Yellow</t>
+  </si>
+  <si>
+    <t>Unwaxed Lemons 10X8</t>
+  </si>
+  <si>
+    <t>Unwaxed 10x8</t>
+  </si>
+  <si>
+    <t>Front 10x8</t>
+  </si>
+  <si>
+    <t>20% off</t>
+  </si>
+  <si>
+    <t>Back 20x4</t>
+  </si>
+  <si>
+    <t>Front 20x4</t>
+  </si>
+  <si>
+    <t>Unwaxed 20x4</t>
+  </si>
+  <si>
+    <t>Unwaxed Lemons 20x4</t>
+  </si>
+  <si>
+    <t>MEP Clementines</t>
+  </si>
+  <si>
+    <t>Mini E/P</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>Clementines EP</t>
+  </si>
+  <si>
+    <t>Easy Peelers</t>
   </si>
 </sst>
 </file>
@@ -130,13 +182,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -438,12 +491,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -515,25 +569,107 @@
         <v>15</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>